<commit_message>
[auto-snapshot] 2026-05-02 16:00 | onda-hompage | 197 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_derma/강서구_피부과.xlsx
+++ b/naver-place-crawler/results_derma/강서구_피부과.xlsx
@@ -417,13 +417,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V10"/>
+  <dimension ref="A1:V9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="29" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="41" customWidth="1" min="7" max="7"/>
@@ -596,7 +596,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -612,7 +612,7 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -621,13 +621,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>17750</v>
+        <v>17960</v>
       </c>
       <c r="Q2" t="n">
-        <v>8772</v>
+        <v>8889</v>
       </c>
       <c r="R2" t="n">
-        <v>26522</v>
+        <v>26849</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -658,38 +658,34 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>프리마피부과의원 강서</t>
+          <t>샤인빔의원 강서</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>kokona1213@naver.com</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>webtick@gmail.com</t>
-        </is>
-      </c>
+          <t>shinebeam_gangseo@naver.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>02-2607-7574</t>
+          <t>02-1544-5236</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>서울특별시 강서구 화곡로 157 로이빌딩 3층</t>
+          <t>서울특별시 강서구 공항대로 247 퀸즈파크나인 C동 3층 상담센터</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.primaderma.co.kr</t>
+          <t>http://gangseo.shinebeam.co.kr/</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -699,7 +695,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -719,13 +715,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>2332</v>
+        <v>2262</v>
       </c>
       <c r="Q3" t="n">
-        <v>2081</v>
+        <v>4255</v>
       </c>
       <c r="R3" t="n">
-        <v>4413</v>
+        <v>6517</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -734,17 +730,17 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>19504262</t>
+          <t>1883636153</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/19504262</t>
+          <t>https://m.place.naver.com/place/1883636153</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -756,34 +752,34 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>블리비의원 발산점</t>
+          <t>뷰티온의원 마곡점</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>gp___e@naver.com</t>
+          <t>beautyon_01@naver.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1833-9986</t>
+          <t>0507-1471-7838</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>서울특별시 강서구 강서로 395 3층(마곡동, 플레이스H)</t>
+          <t>서울특별시 강서구 마곡중앙6로 93 8층 801호, 802호, 803호</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>http://www.velyb.kr/</t>
+          <t>https://gangseo.beautyon.co.kr/</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -804,22 +800,22 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>1791</v>
+        <v>6470</v>
       </c>
       <c r="Q4" t="n">
-        <v>4553</v>
+        <v>7907</v>
       </c>
       <c r="R4" t="n">
-        <v>6344</v>
+        <v>14377</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -828,17 +824,17 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1219387447</t>
+          <t>1134191796</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1219387447</t>
+          <t>https://m.place.naver.com/place/1134191796</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -850,34 +846,34 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>뷰티온의원 마곡점</t>
+          <t>블리비의원 발산점</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>beautyon_01@naver.com</t>
+          <t>gp___e@naver.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0507-1471-7838</t>
+          <t>1833-9986</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>서울특별시 강서구 마곡중앙6로 93 8층 801호, 802호, 803호</t>
+          <t>서울특별시 강서구 강서로 395 3층(마곡동, 플레이스H)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://gangseo.beautyon.co.kr/</t>
+          <t>http://www.velyb.kr/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -898,22 +894,22 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>6406</v>
+        <v>1829</v>
       </c>
       <c r="Q5" t="n">
-        <v>8471</v>
+        <v>4269</v>
       </c>
       <c r="R5" t="n">
-        <v>14877</v>
+        <v>6098</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -922,17 +918,17 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1134191796</t>
+          <t>1219387447</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1134191796</t>
+          <t>https://m.place.naver.com/place/1219387447</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -944,44 +940,44 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>샤인빔의원 강서</t>
+          <t>강서톡스앤필의원</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>shinebeam_gangseo@naver.com</t>
+          <t>toxnfill_gs@naver.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>02-1544-5236</t>
+          <t>02-6958-8688</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>서울특별시 강서구 공항대로 247 퀸즈파크나인 C동 3층 상담센터</t>
+          <t>서울특별시 강서구 공항대로 190 푸리마타워 2층 201호~207호</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>http://gangseo.shinebeam.co.kr/</t>
+          <t>http://www.toxnfill32.com/</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1001,13 +997,13 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>2253</v>
+        <v>457</v>
       </c>
       <c r="Q6" t="n">
-        <v>5253</v>
+        <v>5963</v>
       </c>
       <c r="R6" t="n">
-        <v>7506</v>
+        <v>6420</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1016,17 +1012,17 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1883636153</t>
+          <t>1195059636</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1883636153</t>
+          <t>https://m.place.naver.com/place/1195059636</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1038,44 +1034,44 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>아비쥬의원 강서</t>
+          <t>차앤유의원</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>abijou0@naver.com</t>
+          <t>cnu1357@naver.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1544-0377</t>
+          <t>02-3664-9003</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>서울특별시 강서구 공항대로 236 지하1층</t>
+          <t>서울특별시 강서구 양천로 452 예다인 B동 2층</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://abijouclinicgs.com/</t>
+          <t>http://www.cnuclinic.co.kr/</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1086,22 +1082,22 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>639</v>
+        <v>3191</v>
       </c>
       <c r="Q7" t="n">
-        <v>1615</v>
+        <v>20103</v>
       </c>
       <c r="R7" t="n">
-        <v>2254</v>
+        <v>23294</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1110,17 +1106,17 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1952625367</t>
+          <t>12975400</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1952625367</t>
+          <t>https://m.place.naver.com/place/12975400</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1132,44 +1128,44 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>차앤유의원</t>
+          <t>오빛나의원</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>cnu1357@naver.com</t>
+          <t>ohbitna_clinic@naver.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>02-3664-9003</t>
+          <t>0507-1386-5037</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>서울특별시 강서구 양천로 452 예다인 B동 2층</t>
+          <t>서울특별시 강서구 강서로 380 2층</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>http://www.cnuclinic.co.kr/</t>
+          <t>https://www.ohbitnaclinic.com/</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1180,22 +1176,22 @@
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>3191</v>
+        <v>180</v>
       </c>
       <c r="Q8" t="n">
-        <v>19985</v>
+        <v>186</v>
       </c>
       <c r="R8" t="n">
-        <v>23176</v>
+        <v>366</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1204,17 +1200,17 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>12975400</t>
+          <t>1684351466</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/12975400</t>
+          <t>https://m.place.naver.com/place/1684351466</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>
@@ -1226,34 +1222,34 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>쁘띠케이의원 우장산역</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>petitkclinic@naver.com</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>하이라인피부과의원</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>highlineskin.official@gmail.com</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>02-2065-3075</t>
+          <t>1660-2480</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>서울특별시 강서구 강서로 242 강서힐스테이트 상가동 207호</t>
+          <t>서울특별시 강서구 공항대로 165 원그로브 A동 2층</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>http://petitk.co.kr</t>
+          <t>https://www.highlineskin.com</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1283,13 +1279,13 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>350</v>
+        <v>298</v>
       </c>
       <c r="Q9" t="n">
-        <v>500</v>
+        <v>85</v>
       </c>
       <c r="R9" t="n">
-        <v>850</v>
+        <v>383</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1298,111 +1294,17 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1252972942</t>
+          <t>2048541709</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1252972942</t>
+          <t>https://m.place.naver.com/place/2048541709</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>피부과</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>오라클피부과의원</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>aoracle@naver.com</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>02-2605-1175</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>서울특별시 강서구 화곡로 176-4 화곡메디칼프라자 7층</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>http://www.hkoracle.co.kr/</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P10" t="n">
-        <v>700</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>207</v>
-      </c>
-      <c r="R10" t="n">
-        <v>907</v>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>19515496</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>https://m.place.naver.com/place/19515496</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>2026-04-15</t>
+          <t>2026-05-01</t>
         </is>
       </c>
     </row>

</xml_diff>